<commit_message>
Daily slate 2026-06-24 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-22.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-22.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E2" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F2" t="n">
         <v>136</v>
       </c>
       <c r="G2" t="n">
-        <v>48.9</v>
+        <v>49.1</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F3" t="n">
         <v>40</v>
       </c>
       <c r="G3" t="n">
-        <v>57.9</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>417</v>
+        <v>442</v>
       </c>
       <c r="E4" t="n">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F4" t="n">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="G4" t="n">
-        <v>30</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="5">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F7" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="G7" t="n">
-        <v>54.1</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="8">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E9" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G9" t="n">
-        <v>54.7</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>906</v>
+        <v>998</v>
       </c>
       <c r="E11" t="n">
-        <v>523</v>
+        <v>582</v>
       </c>
       <c r="F11" t="n">
-        <v>383</v>
+        <v>416</v>
       </c>
       <c r="G11" t="n">
-        <v>57.7</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="E12" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="F12" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G12" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G13" t="n">
-        <v>61.7</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>323</v>
+        <v>355</v>
       </c>
       <c r="E14" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F14" t="n">
-        <v>258</v>
+        <v>281</v>
       </c>
       <c r="G14" t="n">
-        <v>20.1</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="15">
@@ -848,13 +848,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>420</v>
+        <v>459</v>
       </c>
       <c r="E15" t="n">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F15" t="n">
-        <v>337</v>
+        <v>368</v>
       </c>
       <c r="G15" t="n">
         <v>19.8</v>
@@ -877,13 +877,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E16" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F16" t="n">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G16" t="n">
         <v>22.6</v>
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4368</v>
+        <v>4759</v>
       </c>
       <c r="E17" t="n">
-        <v>612</v>
+        <v>719</v>
       </c>
       <c r="F17" t="n">
-        <v>3756</v>
+        <v>4040</v>
       </c>
       <c r="G17" t="n">
-        <v>14</v>
+        <v>15.1</v>
       </c>
     </row>
   </sheetData>
@@ -1585,58 +1585,58 @@
         <v>432</v>
       </c>
       <c r="D7" t="n">
-        <v>57.7</v>
+        <v>58.3</v>
       </c>
       <c r="E7" t="n">
-        <v>906</v>
+        <v>998</v>
       </c>
       <c r="F7" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
       <c r="G7" t="n">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="H7" t="n">
-        <v>61.7</v>
+        <v>61.2</v>
       </c>
       <c r="I7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J7" t="n">
-        <v>20.1</v>
+        <v>20.8</v>
       </c>
       <c r="K7" t="n">
-        <v>323</v>
+        <v>355</v>
       </c>
       <c r="L7" t="n">
         <v>19.8</v>
       </c>
       <c r="M7" t="n">
-        <v>420</v>
+        <v>459</v>
       </c>
       <c r="N7" t="n">
         <v>22.6</v>
       </c>
       <c r="O7" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="P7" t="n">
-        <v>14</v>
+        <v>15.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>4368</v>
+        <v>4759</v>
       </c>
       <c r="R7" t="n">
-        <v>48.9</v>
+        <v>49.1</v>
       </c>
       <c r="S7" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="T7" t="n">
-        <v>30</v>
+        <v>31.7</v>
       </c>
       <c r="U7" t="n">
-        <v>417</v>
+        <v>442</v>
       </c>
       <c r="V7" t="n">
         <v>25</v>
@@ -1651,10 +1651,10 @@
         <v>91</v>
       </c>
       <c r="Z7" t="n">
-        <v>57.9</v>
+        <v>58.3</v>
       </c>
       <c r="AA7" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AB7" t="n">
         <v>37.3</v>
@@ -1663,16 +1663,16 @@
         <v>51</v>
       </c>
       <c r="AD7" t="n">
-        <v>54.1</v>
+        <v>52.2</v>
       </c>
       <c r="AE7" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="AF7" t="n">
-        <v>54.7</v>
+        <v>55.7</v>
       </c>
       <c r="AG7" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>